<commit_message>
Validatie van configuratie tabellen aangepast
</commit_message>
<xml_diff>
--- a/config/config - error.xlsx
+++ b/config/config - error.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vrln.sharepoint.com/sites/GGD-ONDZ/PSchijf/Gezondheidsmonitor/Algemeen/Automatisering en R/0. Github/report_excel_to_powerpoint/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ec0ed70858de1434/Bestanden MarSan/10. Coding/report_generator/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="455" documentId="13_ncr:1_{DF16CF3D-75F7-471B-AA95-A327D2E0CD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63DF76CB-7640-430E-8198-781392872C17}"/>
+  <xr:revisionPtr revIDLastSave="456" documentId="13_ncr:1_{DF16CF3D-75F7-471B-AA95-A327D2E0CD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0565397A-8173-4186-AD42-9BD924B9BD0A}"/>
   <bookViews>
-    <workbookView xWindow="49380" yWindow="-5460" windowWidth="15030" windowHeight="12225" activeTab="1" xr2:uid="{340DDFAE-1A83-41FC-A379-531A17E4526A}"/>
+    <workbookView xWindow="18195" yWindow="4260" windowWidth="19605" windowHeight="15345" activeTab="2" xr2:uid="{340DDFAE-1A83-41FC-A379-531A17E4526A}"/>
   </bookViews>
   <sheets>
     <sheet name="reports" sheetId="4" r:id="rId1"/>
     <sheet name="ata" sheetId="7" r:id="rId2"/>
-    <sheet name="dimensions" sheetId="8" r:id="rId3"/>
+    <sheet name="imensions" sheetId="8" r:id="rId3"/>
     <sheet name="slideconfig" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
@@ -1259,8 +1259,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Komma" xfId="4" builtinId="3"/>
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="4" builtinId="3"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{039B6AD3-6FED-4C83-843D-36BA42A5800D}"/>
     <cellStyle name="Standaard 3" xfId="3" xr:uid="{F7250D72-35B9-4D07-B4AB-A751800EFF26}"/>
     <cellStyle name="Standaard 4" xfId="1" xr:uid="{CCC7F1B7-9981-461C-80FF-6B557AD7DF0B}"/>
@@ -1279,7 +1279,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1576,16 +1576,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F0AA7A9-459B-4958-BBC2-94F84CFD8846}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="23.44140625" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="4"/>
+    <col min="1" max="1" width="17.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="8.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>155</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1624,14 +1624,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC43E578-8F83-47C5-8B25-31E9567225DB}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="19" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>147</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>149</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>150</v>
       </c>
@@ -1664,15 +1664,15 @@
         <v>152</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
     </row>
@@ -1686,17 +1686,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF920A0E-36AB-4EC6-823F-965B4C051F80}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="24.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="4"/>
+    <col min="1" max="1" width="19.28515625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>155</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>0</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>0</v>
       </c>
@@ -1810,30 +1810,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF87A273-214F-4086-84B2-968343C1FFDC}">
   <dimension ref="A1:S43"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="56.33203125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" style="17" customWidth="1"/>
-    <col min="5" max="5" width="32.109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="20.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.44140625" style="4" customWidth="1"/>
-    <col min="14" max="14" width="15.109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.109375" style="2" customWidth="1"/>
-    <col min="17" max="18" width="8.88671875" style="2"/>
-    <col min="19" max="19" width="13.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="56.28515625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="17" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" style="2" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.42578125" style="4" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.140625" style="2" customWidth="1"/>
+    <col min="17" max="18" width="8.85546875" style="2"/>
+    <col min="19" max="19" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>35</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>64</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>9</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>15</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>117</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>118</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>119</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>120</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>121</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>122</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>123</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>124</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>125</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>126</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>127</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>128</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>129</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>130</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>131</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>132</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>133</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>134</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>139</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>140</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>141</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>142</v>
       </c>
@@ -3010,7 +3010,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="69" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:19" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>18</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="69" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>56</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="69" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
         <v>68</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>66</v>
       </c>
@@ -3161,7 +3161,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>69</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>96</v>
       </c>
@@ -3235,7 +3235,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>76</v>
       </c>
@@ -3271,7 +3271,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
         <v>77</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>78</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
         <v>79</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>91</v>
       </c>
@@ -3417,7 +3417,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>91</v>
       </c>
@@ -3458,7 +3458,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>92</v>
       </c>
@@ -3497,6 +3497,31 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4e95bed8-6d15-4403-ad70-a53422338dca">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C4EA295FB1FB9547A73C9F5819D6E613" ma:contentTypeVersion="23" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="fb09b8f9996d29818860aca561f17aea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4e95bed8-6d15-4403-ad70-a53422338dca" xmlns:ns3="10d3344f-2d16-43d9-a145-97142f5cb288" xmlns:ns4="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f29125cba2118f3064d103e6e0ba85ce" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3781,32 +3806,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFBB421F-7112-4B85-A662-9379706C03DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4e95bed8-6d15-4403-ad70-a53422338dca"/>
+    <ds:schemaRef ds:uri="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4e95bed8-6d15-4403-ad70-a53422338dca">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0EF40A6-8528-4994-A94E-1AE934020AF5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4DEBE89-047E-4EFF-AFED-68832042A230}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3825,24 +3845,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0EF40A6-8528-4994-A94E-1AE934020AF5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFBB421F-7112-4B85-A662-9379706C03DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4e95bed8-6d15-4403-ad70-a53422338dca"/>
-    <ds:schemaRef ds:uri="d045ab76-3bb7-45f5-ab41-d7b04aa0dc94"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>